<commit_message>
Add M365 assist, dark UI refresh, and Ollama workbook translate.
Integrate M365 auth and knowledge resolution, real-time service status polling,
logic tree vs raw expression compare, and experimental JP translation via Ollama.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pm_test_spec_assistant/output/_pytest_evidence_run/logic_traceability.xlsx
+++ b/pm_test_spec_assistant/output/_pytest_evidence_run/logic_traceability.xlsx
@@ -12187,7 +12187,7 @@
       <c r="B48" s="4" t="n"/>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>or_400618e2</t>
+          <t>or_a47ae205</t>
         </is>
       </c>
       <c r="D48" s="4" t="n">
@@ -12225,12 +12225,12 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>or_400618e2</t>
+          <t>or_a47ae205</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>and_b197d5ba</t>
+          <t>and_1131cdcb</t>
         </is>
       </c>
       <c r="D49" s="4" t="n">
@@ -12268,12 +12268,12 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>and_b197d5ba</t>
+          <t>and_1131cdcb</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>ref_a1b7077b</t>
+          <t>ref_4ca27b50</t>
         </is>
       </c>
       <c r="D50" s="4" t="n">
@@ -12319,12 +12319,12 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>and_b197d5ba</t>
+          <t>and_1131cdcb</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>not_610c2466</t>
+          <t>not_f7a8fe5d</t>
         </is>
       </c>
       <c r="D51" s="4" t="n">
@@ -12370,12 +12370,12 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>not_610c2466</t>
+          <t>not_f7a8fe5d</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>ref_dc7a8e49</t>
+          <t>ref_e5f1555f</t>
         </is>
       </c>
       <c r="D52" s="4" t="n">
@@ -12421,12 +12421,12 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>or_400618e2</t>
+          <t>or_a47ae205</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>and_b54630b3</t>
+          <t>and_34d220f6</t>
         </is>
       </c>
       <c r="D53" s="4" t="n">
@@ -12464,12 +12464,12 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>and_b54630b3</t>
+          <t>and_34d220f6</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>ref_df1b12bb</t>
+          <t>ref_07baf230</t>
         </is>
       </c>
       <c r="D54" s="4" t="n">
@@ -12515,12 +12515,12 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>and_b54630b3</t>
+          <t>and_34d220f6</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>ref_cb14e14e</t>
+          <t>ref_764c75a6</t>
         </is>
       </c>
       <c r="D55" s="4" t="n">
@@ -12567,7 +12567,7 @@
       <c r="B56" s="4" t="n"/>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>and_6a09f9b7</t>
+          <t>and_f0e2ef12</t>
         </is>
       </c>
       <c r="D56" s="4" t="n">
@@ -12605,12 +12605,12 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>and_6a09f9b7</t>
+          <t>and_f0e2ef12</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>ref_df03c9e9</t>
+          <t>ref_aaee1505</t>
         </is>
       </c>
       <c r="D57" s="4" t="n">
@@ -12656,12 +12656,12 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>and_6a09f9b7</t>
+          <t>and_f0e2ef12</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>ref_04f179d5</t>
+          <t>ref_7830958b</t>
         </is>
       </c>
       <c r="D58" s="4" t="n">
@@ -12707,12 +12707,12 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>and_6a09f9b7</t>
+          <t>and_f0e2ef12</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>or_9984d74e</t>
+          <t>or_e283e148</t>
         </is>
       </c>
       <c r="D59" s="4" t="n">
@@ -12750,12 +12750,12 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>or_9984d74e</t>
+          <t>or_e283e148</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>ref_f0ed68a6</t>
+          <t>ref_6f400942</t>
         </is>
       </c>
       <c r="D60" s="4" t="n">
@@ -12801,12 +12801,12 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>or_9984d74e</t>
+          <t>or_e283e148</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>op_a035ec5b</t>
+          <t>op_2b44d71e</t>
         </is>
       </c>
       <c r="D61" s="4" t="n">
@@ -12852,12 +12852,12 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>op_a035ec5b</t>
+          <t>op_2b44d71e</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>ref_13cd77ad</t>
+          <t>ref_30093750</t>
         </is>
       </c>
       <c r="D62" s="4" t="n">
@@ -12903,12 +12903,12 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>or_9984d74e</t>
+          <t>or_e283e148</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>ref_18cfa807</t>
+          <t>ref_573ccf9a</t>
         </is>
       </c>
       <c r="D63" s="4" t="n">
@@ -12954,12 +12954,12 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>or_9984d74e</t>
+          <t>or_e283e148</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>op_c17e6b36</t>
+          <t>op_0fc3cd0d</t>
         </is>
       </c>
       <c r="D64" s="4" t="n">
@@ -13005,12 +13005,12 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>op_c17e6b36</t>
+          <t>op_0fc3cd0d</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>ref_196fa6c1</t>
+          <t>ref_6e3412c2</t>
         </is>
       </c>
       <c r="D65" s="4" t="n">
@@ -13056,12 +13056,12 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>or_9984d74e</t>
+          <t>or_e283e148</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>ref_d66c2571</t>
+          <t>ref_c25165c7</t>
         </is>
       </c>
       <c r="D66" s="4" t="n">
@@ -13108,7 +13108,7 @@
       <c r="B67" s="4" t="n"/>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>and_18d91826</t>
+          <t>and_38a55ddf</t>
         </is>
       </c>
       <c r="D67" s="4" t="n">
@@ -13146,12 +13146,12 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>and_18d91826</t>
+          <t>and_38a55ddf</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>ref_4b104c6d</t>
+          <t>ref_2c5a456e</t>
         </is>
       </c>
       <c r="D68" s="4" t="n">
@@ -13197,12 +13197,12 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>and_18d91826</t>
+          <t>and_38a55ddf</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>ref_6590b775</t>
+          <t>ref_a102dd47</t>
         </is>
       </c>
       <c r="D69" s="4" t="n">
@@ -13248,12 +13248,12 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>and_18d91826</t>
+          <t>and_38a55ddf</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>or_cc358963</t>
+          <t>or_d8552ee3</t>
         </is>
       </c>
       <c r="D70" s="4" t="n">
@@ -13291,12 +13291,12 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>or_cc358963</t>
+          <t>or_d8552ee3</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>ref_aa4b028a</t>
+          <t>ref_a51b5ca8</t>
         </is>
       </c>
       <c r="D71" s="4" t="n">
@@ -13342,12 +13342,12 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>or_cc358963</t>
+          <t>or_d8552ee3</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>ref_2679e743</t>
+          <t>ref_df50a6f9</t>
         </is>
       </c>
       <c r="D72" s="4" t="n">
@@ -13394,7 +13394,7 @@
       <c r="B73" s="4" t="n"/>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>and_c8b630cb</t>
+          <t>and_ed25f8fb</t>
         </is>
       </c>
       <c r="D73" s="4" t="n">
@@ -13432,12 +13432,12 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>and_c8b630cb</t>
+          <t>and_ed25f8fb</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>ref_63aefe8b</t>
+          <t>ref_00bd5ccd</t>
         </is>
       </c>
       <c r="D74" s="4" t="n">
@@ -13483,12 +13483,12 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>and_c8b630cb</t>
+          <t>and_ed25f8fb</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>ref_525b38ed</t>
+          <t>ref_53906bbf</t>
         </is>
       </c>
       <c r="D75" s="4" t="n">
@@ -13534,12 +13534,12 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>and_c8b630cb</t>
+          <t>and_ed25f8fb</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>not_5aa1fc2d</t>
+          <t>not_81e31aee</t>
         </is>
       </c>
       <c r="D76" s="4" t="n">
@@ -13585,12 +13585,12 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>not_5aa1fc2d</t>
+          <t>not_81e31aee</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>ref_82cedba0</t>
+          <t>ref_36faad91</t>
         </is>
       </c>
       <c r="D77" s="4" t="n">
@@ -13636,12 +13636,12 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>and_c8b630cb</t>
+          <t>and_ed25f8fb</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>or_b7c8a1bc</t>
+          <t>or_3df34742</t>
         </is>
       </c>
       <c r="D78" s="4" t="n">
@@ -13679,12 +13679,12 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>or_b7c8a1bc</t>
+          <t>or_3df34742</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>ref_6e6fbf82</t>
+          <t>ref_592fed35</t>
         </is>
       </c>
       <c r="D79" s="4" t="n">
@@ -13730,12 +13730,12 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>or_b7c8a1bc</t>
+          <t>or_3df34742</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>ref_de313db7</t>
+          <t>ref_db9bb636</t>
         </is>
       </c>
       <c r="D80" s="4" t="n">
@@ -13782,7 +13782,7 @@
       <c r="B81" s="4" t="n"/>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>or_9795a242</t>
+          <t>or_63031b5b</t>
         </is>
       </c>
       <c r="D81" s="4" t="n">
@@ -13820,12 +13820,12 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>or_9795a242</t>
+          <t>or_63031b5b</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>and_8fe5ddc3</t>
+          <t>and_3faf1d5c</t>
         </is>
       </c>
       <c r="D82" s="4" t="n">
@@ -13863,12 +13863,12 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>and_8fe5ddc3</t>
+          <t>and_3faf1d5c</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>ref_c3589585</t>
+          <t>ref_1b69b228</t>
         </is>
       </c>
       <c r="D83" s="4" t="n">
@@ -13914,12 +13914,12 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>and_8fe5ddc3</t>
+          <t>and_3faf1d5c</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>not_e2453789</t>
+          <t>not_44d128be</t>
         </is>
       </c>
       <c r="D84" s="4" t="n">
@@ -13965,12 +13965,12 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>not_e2453789</t>
+          <t>not_44d128be</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>ref_be1d17be</t>
+          <t>ref_17c770c8</t>
         </is>
       </c>
       <c r="D85" s="4" t="n">
@@ -14016,12 +14016,12 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>or_9795a242</t>
+          <t>or_63031b5b</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>and_05e146bc</t>
+          <t>and_b5cb4b3b</t>
         </is>
       </c>
       <c r="D86" s="4" t="n">
@@ -14059,12 +14059,12 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>and_05e146bc</t>
+          <t>and_b5cb4b3b</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>ref_cc235960</t>
+          <t>ref_16fa05a5</t>
         </is>
       </c>
       <c r="D87" s="4" t="n">
@@ -14110,12 +14110,12 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>and_05e146bc</t>
+          <t>and_b5cb4b3b</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>ref_a5101e50</t>
+          <t>ref_836e8070</t>
         </is>
       </c>
       <c r="D88" s="4" t="n">
@@ -14162,7 +14162,7 @@
       <c r="B89" s="4" t="n"/>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>and_76f35c60</t>
+          <t>and_47ec2d1c</t>
         </is>
       </c>
       <c r="D89" s="4" t="n">
@@ -14200,12 +14200,12 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>and_76f35c60</t>
+          <t>and_47ec2d1c</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>ref_0b1431ef</t>
+          <t>ref_b692b4f5</t>
         </is>
       </c>
       <c r="D90" s="4" t="n">
@@ -14251,12 +14251,12 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>and_76f35c60</t>
+          <t>and_47ec2d1c</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>ref_e98a3c61</t>
+          <t>ref_00e4f522</t>
         </is>
       </c>
       <c r="D91" s="4" t="n">
@@ -14302,12 +14302,12 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>and_76f35c60</t>
+          <t>and_47ec2d1c</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>or_d8cb5140</t>
+          <t>or_85a49f29</t>
         </is>
       </c>
       <c r="D92" s="4" t="n">
@@ -14345,12 +14345,12 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>or_d8cb5140</t>
+          <t>or_85a49f29</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>ref_d94b2e4d</t>
+          <t>ref_e354e98c</t>
         </is>
       </c>
       <c r="D93" s="4" t="n">
@@ -14396,12 +14396,12 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>or_d8cb5140</t>
+          <t>or_85a49f29</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>op_52965c5b</t>
+          <t>op_1608a685</t>
         </is>
       </c>
       <c r="D94" s="4" t="n">
@@ -14447,12 +14447,12 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>op_52965c5b</t>
+          <t>op_1608a685</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>ref_137b1e40</t>
+          <t>ref_f81a17fb</t>
         </is>
       </c>
       <c r="D95" s="4" t="n">
@@ -14498,12 +14498,12 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>or_d8cb5140</t>
+          <t>or_85a49f29</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>ref_cea2b651</t>
+          <t>ref_52964cf3</t>
         </is>
       </c>
       <c r="D96" s="4" t="n">
@@ -14549,12 +14549,12 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>or_d8cb5140</t>
+          <t>or_85a49f29</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>op_624864bc</t>
+          <t>op_21351268</t>
         </is>
       </c>
       <c r="D97" s="4" t="n">
@@ -14600,12 +14600,12 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>op_624864bc</t>
+          <t>op_21351268</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>ref_102d2ec8</t>
+          <t>ref_984a1cf2</t>
         </is>
       </c>
       <c r="D98" s="4" t="n">
@@ -14651,12 +14651,12 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>or_d8cb5140</t>
+          <t>or_85a49f29</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>ref_8245a972</t>
+          <t>ref_e4e7c6d8</t>
         </is>
       </c>
       <c r="D99" s="4" t="n">
@@ -14703,7 +14703,7 @@
       <c r="B100" s="4" t="n"/>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>and_dcf7928a</t>
+          <t>and_829a8b7e</t>
         </is>
       </c>
       <c r="D100" s="4" t="n">
@@ -14741,12 +14741,12 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>and_dcf7928a</t>
+          <t>and_829a8b7e</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>ref_5bea73c2</t>
+          <t>ref_cd1ab74f</t>
         </is>
       </c>
       <c r="D101" s="4" t="n">
@@ -14792,12 +14792,12 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>and_dcf7928a</t>
+          <t>and_829a8b7e</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>ref_595c6851</t>
+          <t>ref_3e5d7f07</t>
         </is>
       </c>
       <c r="D102" s="4" t="n">
@@ -14843,12 +14843,12 @@
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>and_dcf7928a</t>
+          <t>and_829a8b7e</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>or_04c046ad</t>
+          <t>or_9ce52774</t>
         </is>
       </c>
       <c r="D103" s="4" t="n">
@@ -14886,12 +14886,12 @@
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>or_04c046ad</t>
+          <t>or_9ce52774</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>ref_cdd7c824</t>
+          <t>ref_630cb450</t>
         </is>
       </c>
       <c r="D104" s="4" t="n">
@@ -14937,12 +14937,12 @@
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>or_04c046ad</t>
+          <t>or_9ce52774</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>ref_8e69051c</t>
+          <t>ref_75b453d3</t>
         </is>
       </c>
       <c r="D105" s="4" t="n">
@@ -14989,7 +14989,7 @@
       <c r="B106" s="4" t="n"/>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>and_16ad5ec4</t>
+          <t>and_b798001a</t>
         </is>
       </c>
       <c r="D106" s="4" t="n">
@@ -15027,12 +15027,12 @@
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>and_16ad5ec4</t>
+          <t>and_b798001a</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>ref_0d727e04</t>
+          <t>ref_ab3941bc</t>
         </is>
       </c>
       <c r="D107" s="4" t="n">
@@ -15078,12 +15078,12 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>and_16ad5ec4</t>
+          <t>and_b798001a</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>ref_0f2ff2f7</t>
+          <t>ref_a276f7a1</t>
         </is>
       </c>
       <c r="D108" s="4" t="n">
@@ -15129,12 +15129,12 @@
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>and_16ad5ec4</t>
+          <t>and_b798001a</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>not_9368d3c9</t>
+          <t>not_fc92940b</t>
         </is>
       </c>
       <c r="D109" s="4" t="n">
@@ -15180,12 +15180,12 @@
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>not_9368d3c9</t>
+          <t>not_fc92940b</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>ref_0c249b98</t>
+          <t>ref_d3508609</t>
         </is>
       </c>
       <c r="D110" s="4" t="n">
@@ -15231,12 +15231,12 @@
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>and_16ad5ec4</t>
+          <t>and_b798001a</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>or_ddc6193f</t>
+          <t>or_5f98ea25</t>
         </is>
       </c>
       <c r="D111" s="4" t="n">
@@ -15274,12 +15274,12 @@
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>or_ddc6193f</t>
+          <t>or_5f98ea25</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>ref_826cef47</t>
+          <t>ref_9e7730f9</t>
         </is>
       </c>
       <c r="D112" s="4" t="n">
@@ -15325,12 +15325,12 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>or_ddc6193f</t>
+          <t>or_5f98ea25</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>ref_7ebaa6f9</t>
+          <t>ref_dc91f90a</t>
         </is>
       </c>
       <c r="D113" s="4" t="n">

</xml_diff>